<commit_message>
renumber figures, tweak figure appearances
</commit_message>
<xml_diff>
--- a/1-data/TableS2.xlsx
+++ b/1-data/TableS2.xlsx
@@ -383,13 +383,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C2">
-        <v>0.9541919335307547</v>
+        <v>0.9216376268957175</v>
       </c>
       <c r="D2">
-        <v>2.213890461914766E-88</v>
+        <v>3.81836788233267E-70</v>
       </c>
     </row>
     <row r="3">
@@ -409,10 +409,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>1201</v>
+        <v>1227</v>
       </c>
       <c r="C4">
-        <v>0.9594416630479097</v>
+        <v>0.9387228135179511</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -425,13 +425,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5">
-        <v>0.2033062947937699</v>
+        <v>0.1663862400663275</v>
       </c>
       <c r="D5">
-        <v>0.5998297512556078</v>
+        <v>0.645940111078992</v>
       </c>
     </row>
     <row r="6">
@@ -441,13 +441,13 @@
         </is>
       </c>
       <c r="B6">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="C6">
-        <v>0.9654455693911967</v>
+        <v>0.9422323548501894</v>
       </c>
       <c r="D6">
-        <v>1.180004141562231E-138</v>
+        <v>7.584230320981243E-119</v>
       </c>
     </row>
     <row r="7">
@@ -457,13 +457,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>132</v>
+        <v>218</v>
       </c>
       <c r="C7">
-        <v>0.9114052421198748</v>
+        <v>0.8756782586795234</v>
       </c>
       <c r="D7">
-        <v>5.665071250247359E-52</v>
+        <v>3.18748789630783E-70</v>
       </c>
     </row>
     <row r="8">
@@ -473,13 +473,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="C8">
-        <v>0.8043093959808779</v>
+        <v>0.5996707871205558</v>
       </c>
       <c r="D8">
-        <v>7.374736806967728E-07</v>
+        <v>1.694671799540297E-05</v>
       </c>
     </row>
     <row r="9">
@@ -489,10 +489,10 @@
         </is>
       </c>
       <c r="B9">
-        <v>4022</v>
+        <v>3056</v>
       </c>
       <c r="C9">
-        <v>0.959311916234335</v>
+        <v>0.9703262328300104</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -505,13 +505,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>229</v>
+        <v>253</v>
       </c>
       <c r="C10">
-        <v>0.8353696204565505</v>
+        <v>0.7823336342514898</v>
       </c>
       <c r="D10">
-        <v>6.415893357616495E-61</v>
+        <v>1.581715970714502E-53</v>
       </c>
     </row>
     <row r="11">
@@ -521,13 +521,13 @@
         </is>
       </c>
       <c r="B11">
-        <v>223</v>
+        <v>317</v>
       </c>
       <c r="C11">
-        <v>0.9455641992427937</v>
+        <v>0.9039221983430165</v>
       </c>
       <c r="D11">
-        <v>1.018864287957855E-109</v>
+        <v>3.190678359174575E-118</v>
       </c>
     </row>
     <row r="12">
@@ -540,10 +540,10 @@
         <v>3</v>
       </c>
       <c r="C12">
-        <v>-0.930942731129252</v>
+        <v>-0.9309427311292509</v>
       </c>
       <c r="D12">
-        <v>0.2379750047237237</v>
+        <v>0.2379750047237256</v>
       </c>
     </row>
     <row r="13">
@@ -553,10 +553,10 @@
         </is>
       </c>
       <c r="B13">
-        <v>1198</v>
+        <v>1341</v>
       </c>
       <c r="C13">
-        <v>0.9287776657166942</v>
+        <v>0.8935734518477363</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -579,7 +579,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -589,13 +589,13 @@
         </is>
       </c>
       <c r="B16">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="C16">
-        <v>0.9730854085883262</v>
+        <v>0.9471248568232076</v>
       </c>
       <c r="D16">
-        <v>8.069231247427778E-83</v>
+        <v>1.863096891012936E-74</v>
       </c>
     </row>
     <row r="17">
@@ -615,13 +615,13 @@
         </is>
       </c>
       <c r="B18">
-        <v>368</v>
+        <v>482</v>
       </c>
       <c r="C18">
-        <v>0.911154857477381</v>
+        <v>0.8507395301364136</v>
       </c>
       <c r="D18">
-        <v>5.459846005111924E-143</v>
+        <v>3.471992337371164E-136</v>
       </c>
     </row>
     <row r="19">
@@ -631,13 +631,13 @@
         </is>
       </c>
       <c r="B19">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C19">
-        <v>0.9300968195181253</v>
+        <v>0.9061956845354457</v>
       </c>
       <c r="D19">
-        <v>0.000809802519590829</v>
+        <v>0.0007586301067218109</v>
       </c>
     </row>
     <row r="20">
@@ -647,13 +647,13 @@
         </is>
       </c>
       <c r="B20">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C20">
-        <v>-0.4973511477383292</v>
+        <v>-0.5236280554899425</v>
       </c>
       <c r="D20">
-        <v>0.2560985002635067</v>
+        <v>0.1828999507983859</v>
       </c>
     </row>
     <row r="21">
@@ -663,13 +663,13 @@
         </is>
       </c>
       <c r="B21">
-        <v>312</v>
+        <v>359</v>
       </c>
       <c r="C21">
-        <v>0.9446734577236381</v>
+        <v>0.881268753713105</v>
       </c>
       <c r="D21">
-        <v>4.040108717919057E-152</v>
+        <v>3.014246690139377E-118</v>
       </c>
     </row>
     <row r="22">
@@ -679,13 +679,13 @@
         </is>
       </c>
       <c r="B22">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="C22">
-        <v>0.9797870366767661</v>
+        <v>0.9647992549437189</v>
       </c>
       <c r="D22">
-        <v>1.939150158747291E-114</v>
+        <v>1.640096297997828E-107</v>
       </c>
     </row>
     <row r="23">
@@ -695,13 +695,13 @@
         </is>
       </c>
       <c r="B23">
-        <v>486</v>
+        <v>515</v>
       </c>
       <c r="C23">
-        <v>0.9344832484241239</v>
+        <v>0.9182884190698526</v>
       </c>
       <c r="D23">
-        <v>3.123098622274734E-219</v>
+        <v>1.418069136575424E-208</v>
       </c>
     </row>
     <row r="24">
@@ -721,13 +721,13 @@
         </is>
       </c>
       <c r="B25">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="C25">
-        <v>0.3088885103105353</v>
+        <v>0.3005020552925285</v>
       </c>
       <c r="D25">
-        <v>0.005019971631687562</v>
+        <v>0.001938733171911658</v>
       </c>
     </row>
     <row r="26">
@@ -737,13 +737,13 @@
         </is>
       </c>
       <c r="B26">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="C26">
-        <v>0.9675456044517169</v>
+        <v>0.9104912103069003</v>
       </c>
       <c r="D26">
-        <v>1.163396821897731E-17</v>
+        <v>2.150684791809002E-27</v>
       </c>
     </row>
     <row r="27">
@@ -753,13 +753,7 @@
         </is>
       </c>
       <c r="B27">
-        <v>10</v>
-      </c>
-      <c r="C27">
-        <v>-0.5910041246597486</v>
-      </c>
-      <c r="D27">
-        <v>0.07197791682416642</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28">
@@ -779,13 +773,13 @@
         </is>
       </c>
       <c r="B29">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C29">
-        <v>0.947206576532329</v>
+        <v>0.9167721507122083</v>
       </c>
       <c r="D29">
-        <v>1.535636532779711E-70</v>
+        <v>1.15751380285598E-59</v>
       </c>
     </row>
     <row r="30">
@@ -795,7 +789,7 @@
         </is>
       </c>
       <c r="B30">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>